<commit_message>
Widen autofilter columns, tighten README claims, refresh demo data
- Widen column padding (longest + 5) so the autofilter button no
  longer covers the "Цена, £", "Наличие" and "Рейтинг" headers
- README: fold the link-dedup note into the by-name-collision bullet,
  document that cross-category duplicates aren't removed, align the
  sample run output and incomplete-category wording with the current
  script behavior, clarify that only unrecognized prices are left
  blank, and drop the placeholder Contacts section
- Regenerate output/books.xlsx and output/travel.xlsx with the wider
  columns; replace the README screenshot

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/books.xlsx
+++ b/output/books.xlsx
@@ -442,10 +442,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>

</xml_diff>